<commit_message>
new ylim acous. align + diff excel focus input
</commit_message>
<xml_diff>
--- a/SonoRover One/software/example input/protocol template/template_protocol_input.xlsx
+++ b/SonoRover One/software/example input/protocol template/template_protocol_input.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://radbouduniversiteit-my.sharepoint.com/personal/margely_cornelissen_ru_nl/Documents/Documenten/GitHub/repositories/Radboud-FUS-measurement-kit/SonoRover One/software/example input/protocol template/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://radbouduniversiteit-my.sharepoint.com/personal/margely_cornelissen_ru_nl/Documents/Documenten/Software/repositories/Radboud-FUS-measurement-kit/SonoRover One/software/example input/protocol template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="11_A032F6DB3BF3CF38219BB56A5F687AFCE06D3065" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{458121AD-B514-4998-B182-7B35C481BABD}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{F74D7050-BEF9-4F92-A395-2CEC838FDD51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D66BBE5-F623-4494-AB1D-5B4D493D5B8C}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,15 +36,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
   <si>
     <t>Modulation</t>
-  </si>
-  <si>
-    <t>Square</t>
-  </si>
-  <si>
-    <t>Focus [mm]</t>
   </si>
   <si>
     <t>step_size_x [mm]</t>
@@ -65,22 +59,10 @@
     <t>direction_columns</t>
   </si>
   <si>
-    <t>-x</t>
-  </si>
-  <si>
-    <t>-y</t>
-  </si>
-  <si>
-    <t>+z</t>
-  </si>
-  <si>
     <t>Corresponding value</t>
   </si>
   <si>
     <t>Coordinates based on excel file or parameters on the right?</t>
-  </si>
-  <si>
-    <t>Path and filename of Isppa to Global power conversion excel</t>
   </si>
   <si>
     <t>Path and filename of coordinate excel</t>
@@ -92,25 +74,10 @@
     <t>Pulse Repetition Frequency [Hz]</t>
   </si>
   <si>
-    <t>Pulse Train Duration [ms]</t>
-  </si>
-  <si>
     <t>Pulse duration [us]</t>
   </si>
   <si>
-    <t>Coordinate excel file</t>
-  </si>
-  <si>
     <t>Ramp duration [us]</t>
-  </si>
-  <si>
-    <t>Ramp duration step size [us]</t>
-  </si>
-  <si>
-    <t>Isppa [W/cm2], Global power [mW] or Amplitude [%]</t>
-  </si>
-  <si>
-    <t>Amplitude [%] (fill in 'Corresponding value')</t>
   </si>
   <si>
     <t>max. + x [mm] w.r.t. relative zero</t>
@@ -131,13 +98,49 @@
     <t>max. - z [mm] w.r.t. relative zero</t>
   </si>
   <si>
-    <t>Sequence</t>
+    <t>Sequence number</t>
   </si>
   <si>
-    <t>C:\Temp\Characterization_input\250_26_203.xlsx</t>
+    <t>Rectangular - no ramping</t>
+  </si>
+  <si>
+    <t>Dephasing degree (0 = no dephasing) CURRENLTY ONLY APPLICABLE FOR IGT DS</t>
+  </si>
+  <si>
+    <t>Tag</t>
+  </si>
+  <si>
+    <t>SC - Global power [mW] or IGT - Max. pressure in free water [Mpa], Voltage [V] or Amplitude [%]</t>
+  </si>
+  <si>
+    <t>Acoustical alignment test</t>
+  </si>
+  <si>
+    <t>SC - Global power [mW] (fill in 'Corresponding value')</t>
+  </si>
+  <si>
+    <t>Coordinate excel file</t>
   </si>
   <si>
     <t>C:\Temp\Radboud-FUS-measurement-kit\SonoRover One\software\example input\coordinate templates\1D\Axial_0_01_140mm\Axial_0_01_140mm.csv</t>
+  </si>
+  <si>
+    <t>+z</t>
+  </si>
+  <si>
+    <t>-x</t>
+  </si>
+  <si>
+    <t>-y</t>
+  </si>
+  <si>
+    <t>Focus definition</t>
+  </si>
+  <si>
+    <t>Focus value [mm]</t>
+  </si>
+  <si>
+    <t>Focus wrt mid bowl [mm]</t>
   </si>
 </sst>
 </file>
@@ -219,7 +222,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standaard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -262,8 +265,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="29925434" y="4634441"/>
-          <a:ext cx="6755422" cy="3705954"/>
+          <a:off x="27747384" y="5434541"/>
+          <a:ext cx="7079272" cy="3705954"/>
           <a:chOff x="1109936" y="2363691"/>
           <a:chExt cx="6875015" cy="3645629"/>
         </a:xfrm>
@@ -6975,112 +6978,113 @@
   <dimension ref="A1:Z18"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.25" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.25" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="28.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="26.625" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="22.875" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="33.75" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="16.5" style="3" customWidth="1"/>
+    <col min="4" max="4" width="21.75" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17.25" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="28.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="26.625" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="33.375" style="4" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="18.75" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="54" style="4" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="10.625" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="22.25" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.25" style="3" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="52.75" style="3" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="32.75" style="4" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="28" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="27.625" style="3" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="28.125" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="27.75" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="27.875" style="3" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="27.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="32.375" style="4" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="29.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="29" style="3" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="29.625" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="29.125" style="3" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="29.25" style="3" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="28.875" style="3" bestFit="1" customWidth="1"/>
     <col min="21" max="21" width="14.125" style="3" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="13.875" style="3" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="16.875" style="3" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="15.625" style="3" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="15.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="15.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="15.625" style="3" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="15.375" style="3" bestFit="1" customWidth="1"/>
     <col min="27" max="16384" width="11" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="31.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" ht="94.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>21</v>
+      <c r="E1" s="1" t="s">
+        <v>13</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>22</v>
+      <c r="F1" s="1" t="s">
+        <v>12</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="N1" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="O1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="S1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>17</v>
+      <c r="U1" s="1" t="s">
+        <v>4</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>16</v>
+      <c r="V1" s="1" t="s">
+        <v>5</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>18</v>
+      <c r="W1" s="1" t="s">
+        <v>6</v>
       </c>
-      <c r="I1" s="7" t="s">
-        <v>23</v>
+      <c r="X1" s="1" t="s">
+        <v>1</v>
       </c>
-      <c r="J1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="K1" s="7" t="s">
-        <v>14</v>
-      </c>
-      <c r="L1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="N1" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="P1" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q1" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="R1" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="X1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>3</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>5</v>
       </c>
     </row>
     <row r="2" spans="1:26" ht="78.75" x14ac:dyDescent="0.25">
@@ -7088,44 +7092,44 @@
         <v>1</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="C2" s="3">
         <v>0</v>
       </c>
-      <c r="D2" s="3">
+      <c r="D2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="E2" s="3">
         <v>0</v>
       </c>
-      <c r="E2" s="3">
-        <v>30</v>
-      </c>
       <c r="F2" s="3">
-        <v>5</v>
+        <v>250</v>
       </c>
       <c r="G2" s="3">
-        <f>(1/F2)*1000</f>
-        <v>200</v>
+        <f>1/H2*1000</f>
+        <v>50</v>
       </c>
       <c r="H2" s="3">
-        <v>200</v>
+        <v>20</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="J2" s="3">
-        <v>40</v>
+        <v>0</v>
       </c>
-      <c r="K2" s="4" t="s">
-        <v>32</v>
+      <c r="K2" s="3" t="s">
+        <v>34</v>
       </c>
       <c r="L2" s="3">
         <v>44</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="O2" s="3">
         <v>25</v>
@@ -7146,13 +7150,13 @@
         <v>0</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="V2" s="5" t="s">
-        <v>9</v>
+        <v>30</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>10</v>
+        <v>31</v>
       </c>
       <c r="X2" s="3">
         <v>5</v>
@@ -7274,7 +7278,7 @@
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <dataValidations count="4">
+  <dataValidations count="6">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2:W1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"'+x,'-x,'+y,'-y,'+z,'-z"</formula1>
     </dataValidation>
@@ -7282,10 +7286,16 @@
       <formula1>"Coordinate excel file, Parameters on the right"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1048576" xr:uid="{00000000-0002-0000-0000-000002000000}">
-      <formula1>"Amplitude [%] (fill in 'Corresponding value'),Global power [mW] (fill in 'Corresponding value'),Isppa [W/cm2] (fill in 'Corresponding value' and 'Excel path and filename of Isppa to Global power conversion table'),"</formula1>
+      <formula1>"SC - Global power [mW] (fill in 'Corresponding value'),IGT - Max. pressure in free water [MPa] (fill in 'Corresponding value'),IGT - Voltage [V] (fill in 'Corresponding value'), IGT - Amplitude [%] (fill in 'Corresponding value'),"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B1048576" xr:uid="{00000000-0002-0000-0000-000003000000}">
-      <formula1>"Square,Linear,Tukey,"</formula1>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D1048576" xr:uid="{00000000-0002-0000-0000-000003000000}">
+      <formula1>"Rectangular - no ramping,Linear,Tukey,"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3:K1048576" xr:uid="{278077B7-8E83-470A-A046-016613484199}">
+      <formula1>"Focus wrt exit plane [mm]; Focus wrt mid bowl [mm]"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2" xr:uid="{E821554A-EEDB-4C5D-AEBD-3CA955F53F0B}">
+      <formula1>"Focus wrt exit plane [mm], Focus wrt mid bowl [mm]"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
improved template + power assignment
</commit_message>
<xml_diff>
--- a/SonoRover One/software/example input/protocol template/template_protocol_input.xlsx
+++ b/SonoRover One/software/example input/protocol template/template_protocol_input.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://radbouduniversiteit-my.sharepoint.com/personal/margely_cornelissen_ru_nl/Documents/Documenten/Software/repositories/Radboud-FUS-measurement-kit/SonoRover One/software/example input/protocol template/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitLab\Radboud-FUS-measurement-kit\SonoRover One\software\example input\protocol template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="15" documentId="13_ncr:1_{F74D7050-BEF9-4F92-A395-2CEC838FDD51}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1D66BBE5-F623-4494-AB1D-5B4D493D5B8C}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -104,25 +103,13 @@
     <t>Rectangular - no ramping</t>
   </si>
   <si>
-    <t>Dephasing degree (0 = no dephasing) CURRENLTY ONLY APPLICABLE FOR IGT DS</t>
-  </si>
-  <si>
     <t>Tag</t>
   </si>
   <si>
     <t>SC - Global power [mW] or IGT - Max. pressure in free water [Mpa], Voltage [V] or Amplitude [%]</t>
   </si>
   <si>
-    <t>Acoustical alignment test</t>
-  </si>
-  <si>
-    <t>SC - Global power [mW] (fill in 'Corresponding value')</t>
-  </si>
-  <si>
     <t>Coordinate excel file</t>
-  </si>
-  <si>
-    <t>C:\Temp\Radboud-FUS-measurement-kit\SonoRover One\software\example input\coordinate templates\1D\Axial_0_01_140mm\Axial_0_01_140mm.csv</t>
   </si>
   <si>
     <t>+z</t>
@@ -142,11 +129,23 @@
   <si>
     <t>Focus wrt mid bowl [mm]</t>
   </si>
+  <si>
+    <t>IGT - Amplitude [%] (fill in 'Corresponding value')</t>
+  </si>
+  <si>
+    <t>H:\Hydrophone measurements\!Coordinate Templates\1D\Axial_0_05_140mm\Axial_0_05_140mm.csv</t>
+  </si>
+  <si>
+    <t>Dephasing degree (None = no dephasing) CURRENTLY ONLY APPLICABLE FOR IGT DS</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -265,7 +264,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="27747384" y="5434541"/>
+          <a:off x="27747384" y="5231341"/>
           <a:ext cx="7079272" cy="3705954"/>
           <a:chOff x="1109936" y="2363691"/>
           <a:chExt cx="6875015" cy="3645629"/>
@@ -6974,7 +6973,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Z18"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
@@ -7012,10 +7011,10 @@
         <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C1" s="7" t="s">
-        <v>22</v>
+        <v>33</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>0</v>
@@ -7033,16 +7032,16 @@
         <v>10</v>
       </c>
       <c r="I1" s="7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="J1" s="1" t="s">
         <v>7</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>8</v>
@@ -7087,15 +7086,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:26" ht="78.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" ht="63" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" s="3">
-        <v>0</v>
+      <c r="C2" s="3" t="s">
+        <v>34</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>21</v>
@@ -7114,22 +7110,22 @@
         <v>20</v>
       </c>
       <c r="I2" s="4" t="s">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="J2" s="3">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="K2" s="3" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="L2" s="3">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="M2" s="3" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="O2" s="3">
         <v>25</v>
@@ -7150,13 +7146,13 @@
         <v>0</v>
       </c>
       <c r="U2" s="5" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="V2" s="5" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="W2" s="5" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="X2" s="3">
         <v>5</v>
@@ -7279,22 +7275,22 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2:W1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2:W1048576">
       <formula1>"'+x,'-x,'+y,'-y,'+z,'-z"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:M1048576" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:M1048576">
       <formula1>"Coordinate excel file, Parameters on the right"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1048576" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1048576">
       <formula1>"SC - Global power [mW] (fill in 'Corresponding value'),IGT - Max. pressure in free water [MPa] (fill in 'Corresponding value'),IGT - Voltage [V] (fill in 'Corresponding value'), IGT - Amplitude [%] (fill in 'Corresponding value'),"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D1048576" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D1048576">
       <formula1>"Rectangular - no ramping,Linear,Tukey,"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3:K1048576" xr:uid="{278077B7-8E83-470A-A046-016613484199}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3:K1048576">
       <formula1>"Focus wrt exit plane [mm]; Focus wrt mid bowl [mm]"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2" xr:uid="{E821554A-EEDB-4C5D-AEBD-3CA955F53F0B}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2">
       <formula1>"Focus wrt exit plane [mm], Focus wrt mid bowl [mm]"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7314,17 +7310,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9cb83fc2-d77f-46b4-9581-c00b781f61fd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8754a512-6dec-483d-b5c6-7cffcc0d02c1" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C12600718C676640B862E0AA4EBA4F75" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5b5271ce1c64dd6d8fbb2a683be13c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9cb83fc2-d77f-46b4-9581-c00b781f61fd" xmlns:ns3="8754a512-6dec-483d-b5c6-7cffcc0d02c1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3472f45d873750127c69500d0e5c45f1" ns2:_="" ns3:_="">
     <xsd:import namespace="9cb83fc2-d77f-46b4-9581-c00b781f61fd"/>
@@ -7547,6 +7532,17 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9cb83fc2-d77f-46b4-9581-c00b781f61fd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8754a512-6dec-483d-b5c6-7cffcc0d02c1" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C755C0B-1A1A-4CAB-AAB3-F18FC1BEB5C4}">
   <ds:schemaRefs>
@@ -7556,17 +7552,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{363ED61F-1B79-49C7-A484-F44EFFCDAAF2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9cb83fc2-d77f-46b4-9581-c00b781f61fd"/>
-    <ds:schemaRef ds:uri="8754a512-6dec-483d-b5c6-7cffcc0d02c1"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3099BEFB-1261-4A7B-B1BD-10B30D1875E1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7583,4 +7568,15 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{363ED61F-1B79-49C7-A484-F44EFFCDAAF2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9cb83fc2-d77f-46b4-9581-c00b781f61fd"/>
+    <ds:schemaRef ds:uri="8754a512-6dec-483d-b5c6-7cffcc0d02c1"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
#45 bring dephasing/setting phases to front-end #45
</commit_message>
<xml_diff>
--- a/SonoRover One/software/example input/protocol template/template_protocol_input.xlsx
+++ b/SonoRover One/software/example input/protocol template/template_protocol_input.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\GitLab\Radboud-FUS-measurement-kit\SonoRover One\software\example input\protocol template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://radbouduniversiteit-my.sharepoint.com/personal/margely_cornelissen_ru_nl/Documents/Documenten/Software/repositories/Radboud-FUS-measurement-kit/SonoRover One/software/example input/protocol template/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="63" documentId="11_A0C2F65C2FAEDEC4F639B37A11697A31A069101E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01B23795-19A4-4A7A-9607-5898F3B7E23B}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="40">
   <si>
     <t>Modulation</t>
   </si>
@@ -127,25 +128,82 @@
     <t>Focus value [mm]</t>
   </si>
   <si>
-    <t>Focus wrt mid bowl [mm]</t>
-  </si>
-  <si>
     <t>IGT - Amplitude [%] (fill in 'Corresponding value')</t>
   </si>
   <si>
     <t>H:\Hydrophone measurements\!Coordinate Templates\1D\Axial_0_05_140mm\Axial_0_05_140mm.csv</t>
   </si>
   <si>
-    <t>Dephasing degree (None = no dephasing) CURRENTLY ONLY APPLICABLE FOR IGT DS</t>
+    <t>None</t>
   </si>
   <si>
-    <t>None</t>
+    <t>[0, 90, 180, 270]</t>
+  </si>
+  <si>
+    <t>[90]</t>
+  </si>
+  <si>
+    <t>Focus wrt exit plane [mm]</t>
+  </si>
+  <si>
+    <t>Regular use of focus</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Dephasing with equal degrees using focus</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+ One value (&gt;0) is the degree of dephasing, for example [90] with 4 elements: 1 elem: 0 dephasing, 2 elem: 90 dephasing, 3 elem: 180 dephasing, 4 elem: 270 dephasing. These values will be extracted from the phases calculated with the set focus.</t>
+    </r>
+  </si>
+  <si>
+    <t>(De)phase array [degree] (None = no (de)phasing) ONLY FOR IGT DS</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Override phases</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> 
+When the amount of values match the amount of elements, it will override the calculated phases based on the set focus. Set focus is still required for IGT conversion equations.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -264,7 +322,7 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="27747384" y="5231341"/>
+          <a:off x="29900034" y="7028391"/>
           <a:ext cx="7079272" cy="3705954"/>
           <a:chOff x="1109936" y="2363691"/>
           <a:chExt cx="6875015" cy="3645629"/>
@@ -6973,22 +7031,22 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z18"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="16.5" style="3" customWidth="1"/>
-    <col min="4" max="4" width="21.75" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="17.625" style="3" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="17.25" style="3" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="28.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="26.625" style="3" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="33.375" style="4" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="18.75" style="3" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="22.25" style="3" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.25" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="38.875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="21.75" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.25" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="28.5" style="3" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="26.625" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="33.375" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.75" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="22.25" style="3" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="15.25" style="3" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="16.5" style="3" customWidth="1"/>
     <col min="13" max="13" width="52.75" style="3" bestFit="1" customWidth="1"/>
     <col min="14" max="14" width="32.375" style="4" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="29.5" style="3" bestFit="1" customWidth="1"/>
@@ -7006,42 +7064,42 @@
     <col min="27" max="16384" width="11" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="94.5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" ht="63" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="7" t="s">
-        <v>33</v>
+      <c r="C1" s="1" t="s">
+        <v>0</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="H1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I1" s="7" t="s">
+      <c r="H1" s="7" t="s">
         <v>23</v>
       </c>
+      <c r="I1" s="1" t="s">
+        <v>7</v>
+      </c>
       <c r="J1" s="1" t="s">
-        <v>7</v>
+        <v>28</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="L1" s="1" t="s">
         <v>29</v>
+      </c>
+      <c r="L1" s="7" t="s">
+        <v>38</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>8</v>
@@ -7090,42 +7148,45 @@
       <c r="A2" s="3">
         <v>1</v>
       </c>
+      <c r="B2" s="1" t="s">
+        <v>36</v>
+      </c>
       <c r="C2" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="D2" s="3" t="s">
         <v>21</v>
       </c>
+      <c r="D2" s="3">
+        <v>0</v>
+      </c>
       <c r="E2" s="3">
-        <v>0</v>
+        <v>250</v>
       </c>
       <c r="F2" s="3">
-        <v>250</v>
+        <f>1/G2*1000</f>
+        <v>50</v>
       </c>
       <c r="G2" s="3">
-        <f>1/H2*1000</f>
+        <v>20</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I2" s="3">
+        <v>20</v>
+      </c>
+      <c r="J2" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K2" s="3">
         <v>50</v>
       </c>
-      <c r="H2" s="3">
-        <v>20</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="J2" s="3">
-        <v>20</v>
-      </c>
-      <c r="K2" s="3" t="s">
-        <v>30</v>
-      </c>
-      <c r="L2" s="3">
-        <v>50</v>
+      <c r="L2" s="3" t="s">
+        <v>32</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="O2" s="3">
         <v>25</v>
@@ -7164,15 +7225,167 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="U3" s="5"/>
-      <c r="V3" s="5"/>
-      <c r="W3" s="5"/>
+    <row r="3" spans="1:26" ht="110.25" x14ac:dyDescent="0.25">
+      <c r="A3" s="3">
+        <v>2</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="3">
+        <v>0</v>
+      </c>
+      <c r="E3" s="3">
+        <v>250</v>
+      </c>
+      <c r="F3" s="3">
+        <f>1/G3*1000</f>
+        <v>50</v>
+      </c>
+      <c r="G3" s="3">
+        <v>20</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I3" s="3">
+        <v>20</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K3" s="3">
+        <v>40</v>
+      </c>
+      <c r="L3" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="M3" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="N3" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="O3" s="3">
+        <v>25</v>
+      </c>
+      <c r="P3" s="3">
+        <v>25</v>
+      </c>
+      <c r="Q3" s="3">
+        <v>25</v>
+      </c>
+      <c r="R3" s="3">
+        <v>25</v>
+      </c>
+      <c r="S3" s="3">
+        <v>5</v>
+      </c>
+      <c r="T3" s="3">
+        <v>0</v>
+      </c>
+      <c r="U3" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="V3" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="W3" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="X3" s="3">
+        <v>5</v>
+      </c>
+      <c r="Y3" s="3">
+        <v>5</v>
+      </c>
+      <c r="Z3" s="3">
+        <v>5</v>
+      </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
-      <c r="U4" s="5"/>
-      <c r="V4" s="5"/>
-      <c r="W4" s="5"/>
+    <row r="4" spans="1:26" ht="94.5" x14ac:dyDescent="0.25">
+      <c r="A4" s="3">
+        <v>3</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="3">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3">
+        <v>250</v>
+      </c>
+      <c r="F4" s="3">
+        <f>1/G4*1000</f>
+        <v>50</v>
+      </c>
+      <c r="G4" s="3">
+        <v>20</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I4" s="3">
+        <v>20</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="K4" s="3">
+        <v>30</v>
+      </c>
+      <c r="L4" s="3" t="s">
+        <v>33</v>
+      </c>
+      <c r="M4" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="N4" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="O4" s="3">
+        <v>25</v>
+      </c>
+      <c r="P4" s="3">
+        <v>25</v>
+      </c>
+      <c r="Q4" s="3">
+        <v>25</v>
+      </c>
+      <c r="R4" s="3">
+        <v>25</v>
+      </c>
+      <c r="S4" s="3">
+        <v>5</v>
+      </c>
+      <c r="T4" s="3">
+        <v>0</v>
+      </c>
+      <c r="U4" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="V4" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="W4" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="X4" s="3">
+        <v>5</v>
+      </c>
+      <c r="Y4" s="3">
+        <v>5</v>
+      </c>
+      <c r="Z4" s="3">
+        <v>5</v>
+      </c>
     </row>
     <row r="5" spans="1:26" x14ac:dyDescent="0.25">
       <c r="U5" s="5"/>
@@ -7274,23 +7487,20 @@
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
-  <dataValidations count="6">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2:W1048576">
+  <dataValidations count="5">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2:W1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"'+x,'-x,'+y,'-y,'+z,'-z"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:M1048576" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Coordinate excel file, Parameters on the right"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="I2:I1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H1048576" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"SC - Global power [mW] (fill in 'Corresponding value'),IGT - Max. pressure in free water [MPa] (fill in 'Corresponding value'),IGT - Voltage [V] (fill in 'Corresponding value'), IGT - Amplitude [%] (fill in 'Corresponding value'),"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="D2:D1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Rectangular - no ramping,Linear,Tukey,"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3:K1048576">
-      <formula1>"Focus wrt exit plane [mm]; Focus wrt mid bowl [mm]"</formula1>
-    </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K2">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J1048576" xr:uid="{00000000-0002-0000-0000-000005000000}">
       <formula1>"Focus wrt exit plane [mm], Focus wrt mid bowl [mm]"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
debugging for new release
</commit_message>
<xml_diff>
--- a/SonoRover One/software/example input/protocol template/template_protocol_input.xlsx
+++ b/SonoRover One/software/example input/protocol template/template_protocol_input.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28129"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://radbouduniversiteit-my.sharepoint.com/personal/margely_cornelissen_ru_nl/Documents/Documenten/Software/repositories/Radboud-FUS-measurement-kit/SonoRover One/software/example input/protocol template/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Operator\Documents\GitHub\Radboud-FUS-measurement-kit\SonoRover One\software\example input\protocol template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="11_A0C2F65C2FAEDEC4F639B37A11697A31A069101E" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{01B23795-19A4-4A7A-9607-5898F3B7E23B}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -131,9 +130,6 @@
     <t>IGT - Amplitude [%] (fill in 'Corresponding value')</t>
   </si>
   <si>
-    <t>H:\Hydrophone measurements\!Coordinate Templates\1D\Axial_0_05_140mm\Axial_0_05_140mm.csv</t>
-  </si>
-  <si>
     <t>None</t>
   </si>
   <si>
@@ -199,11 +195,14 @@
 When the amount of values match the amount of elements, it will override the calculated phases based on the set focus. Set focus is still required for IGT conversion equations.</t>
     </r>
   </si>
+  <si>
+    <t>Z:\Hydrophone measurements\!Coordinate Templates\1D\Axial_0_05_140mm\Axial_0_05_140mm.csv</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -7031,7 +7030,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:Z18"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
@@ -7099,7 +7098,7 @@
         <v>29</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>8</v>
@@ -7149,7 +7148,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>21</v>
@@ -7174,19 +7173,19 @@
         <v>20</v>
       </c>
       <c r="J2" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K2" s="3">
         <v>50</v>
       </c>
       <c r="L2" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="O2" s="3">
         <v>25</v>
@@ -7230,7 +7229,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>21</v>
@@ -7255,19 +7254,19 @@
         <v>20</v>
       </c>
       <c r="J3" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K3" s="3">
         <v>40</v>
       </c>
       <c r="L3" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="M3" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="O3" s="3">
         <v>25</v>
@@ -7311,7 +7310,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>21</v>
@@ -7336,19 +7335,19 @@
         <v>20</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="K4" s="3">
         <v>30</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>24</v>
       </c>
       <c r="N4" s="4" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="O4" s="3">
         <v>25</v>
@@ -7488,19 +7487,19 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2:W1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2:W1048576">
       <formula1>"'+x,'-x,'+y,'-y,'+z,'-z"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:M1048576" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:M1048576">
       <formula1>"Coordinate excel file, Parameters on the right"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H1048576" xr:uid="{00000000-0002-0000-0000-000002000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H1048576">
       <formula1>"SC - Global power [mW] (fill in 'Corresponding value'),IGT - Max. pressure in free water [MPa] (fill in 'Corresponding value'),IGT - Voltage [V] (fill in 'Corresponding value'), IGT - Amplitude [%] (fill in 'Corresponding value'),"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576" xr:uid="{00000000-0002-0000-0000-000003000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576">
       <formula1>"Rectangular - no ramping,Linear,Tukey,"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J1048576" xr:uid="{00000000-0002-0000-0000-000005000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J1048576">
       <formula1>"Focus wrt exit plane [mm], Focus wrt mid bowl [mm]"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7520,6 +7519,17 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9cb83fc2-d77f-46b4-9581-c00b781f61fd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8754a512-6dec-483d-b5c6-7cffcc0d02c1" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C12600718C676640B862E0AA4EBA4F75" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5b5271ce1c64dd6d8fbb2a683be13c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9cb83fc2-d77f-46b4-9581-c00b781f61fd" xmlns:ns3="8754a512-6dec-483d-b5c6-7cffcc0d02c1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3472f45d873750127c69500d0e5c45f1" ns2:_="" ns3:_="">
     <xsd:import namespace="9cb83fc2-d77f-46b4-9581-c00b781f61fd"/>
@@ -7742,17 +7752,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9cb83fc2-d77f-46b4-9581-c00b781f61fd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8754a512-6dec-483d-b5c6-7cffcc0d02c1" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C755C0B-1A1A-4CAB-AAB3-F18FC1BEB5C4}">
   <ds:schemaRefs>
@@ -7762,6 +7761,17 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{363ED61F-1B79-49C7-A484-F44EFFCDAAF2}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="9cb83fc2-d77f-46b4-9581-c00b781f61fd"/>
+    <ds:schemaRef ds:uri="8754a512-6dec-483d-b5c6-7cffcc0d02c1"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3099BEFB-1261-4A7B-B1BD-10B30D1875E1}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7778,15 +7788,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{363ED61F-1B79-49C7-A484-F44EFFCDAAF2}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="9cb83fc2-d77f-46b4-9581-c00b781f61fd"/>
-    <ds:schemaRef ds:uri="8754a512-6dec-483d-b5c6-7cffcc0d02c1"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
#58 Handle setting amplitude or voltage per element for IGT equipment
</commit_message>
<xml_diff>
--- a/SonoRover One/software/example input/protocol template/template_protocol_input.xlsx
+++ b/SonoRover One/software/example input/protocol template/template_protocol_input.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="7" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Operator\Documents\GitHub\Radboud-FUS-measurement-kit\SonoRover One\software\example input\protocol template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://radbouduniversiteit-my.sharepoint.com/personal/margely_cornelissen_ru_nl/Documents/Documenten/Software/repositories/Radboud-FUS-measurement-kit/SonoRover One/software/example input/protocol template/"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="15" documentId="11_3CF2DF2D9B157EEC43CAA21843458A6B78AB3715" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9C7582D8-672B-4319-A15A-185621C0FEE1}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -35,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="44">
   <si>
     <t>Modulation</t>
   </si>
@@ -145,31 +146,13 @@
     <t>Regular use of focus</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Dephasing with equal degrees using focus</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> 
- One value (&gt;0) is the degree of dephasing, for example [90] with 4 elements: 1 elem: 0 dephasing, 2 elem: 90 dephasing, 3 elem: 180 dephasing, 4 elem: 270 dephasing. These values will be extracted from the phases calculated with the set focus.</t>
-    </r>
+    <t>(De)phase array [degree] (None = no (de)phasing) ONLY FOR IGT DS</t>
   </si>
   <si>
-    <t>(De)phase array [degree] (None = no (de)phasing) ONLY FOR IGT DS</t>
+    <t>Z:\Hydrophone measurements\!Coordinate Templates\1D\Axial_0_05_140mm\Axial_0_05_140mm.csv</t>
+  </si>
+  <si>
+    <t>Regular use of amplitude or voltage</t>
   </si>
   <si>
     <r>
@@ -181,7 +164,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>Override phases</t>
+      <t>Dephasing with equal degrees using focus (IGT only)</t>
     </r>
     <r>
       <rPr>
@@ -191,18 +174,90 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> 
+      <t xml:space="preserve">
+ One value (&gt;0) is the degree of dephasing, for example [90] with 4 elements: 1 elem: 0 dephasing, 2 elem: 90 dephasing, 3 elem: 180 dephasing, 4 elem: 270 dephasing. These values will be extracted from the phases calculated with the set focus.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Dephasing with equal degrees using focus (IGT only)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+ One value (&gt;0) is the degree of dephasing, for example [90] with 4 elements: 1 elem: 0 dephasing, D202 elem: 90 dephasing, 3 elem: 180 dephasing, 4 elem: 270 dephasing. These values will be extracted from the phases calculated with the set focus.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Override phases (IGT only)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
 When the amount of values match the amount of elements, it will override the calculated phases based on the set focus. Set focus is still required for IGT conversion equations.</t>
     </r>
   </si>
   <si>
-    <t>Z:\Hydrophone measurements\!Coordinate Templates\1D\Axial_0_05_140mm\Axial_0_05_140mm.csv</t>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Defining amplitude or voltages per element (IGT only)</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+When the amount of values match the amount of elements, it will set a different amplitude or voltage per element. If IGT conversion equations apply, they don't apply in this case so pressure will not be calculated.</t>
+    </r>
+  </si>
+  <si>
+    <t>[20, 0, 0, 0, 0, 0, 0, 0, 0, 0]</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -321,8 +376,8 @@
       </xdr:nvGrpSpPr>
       <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="29900034" y="7028391"/>
-          <a:ext cx="7079272" cy="3705954"/>
+          <a:off x="29900034" y="9219141"/>
+          <a:ext cx="7079272" cy="7103204"/>
           <a:chOff x="1109936" y="2363691"/>
           <a:chExt cx="6875015" cy="3645629"/>
         </a:xfrm>
@@ -7030,8 +7085,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Z18"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:Z20"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5" style="3" bestFit="1" customWidth="1"/>
@@ -7098,7 +7153,7 @@
         <v>29</v>
       </c>
       <c r="L1" s="7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="M1" s="1" t="s">
         <v>8</v>
@@ -7185,7 +7240,7 @@
         <v>24</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="O2" s="3">
         <v>25</v>
@@ -7224,12 +7279,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:26" ht="110.25" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" ht="126" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>21</v>
@@ -7266,7 +7321,7 @@
         <v>24</v>
       </c>
       <c r="N3" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="O3" s="3">
         <v>25</v>
@@ -7310,7 +7365,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="C4" s="3" t="s">
         <v>21</v>
@@ -7347,7 +7402,7 @@
         <v>24</v>
       </c>
       <c r="N4" s="4" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="O4" s="3">
         <v>25</v>
@@ -7386,12 +7441,98 @@
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" ht="63" x14ac:dyDescent="0.25">
+      <c r="A5" s="3">
+        <v>4</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="3">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3">
+        <v>250</v>
+      </c>
+      <c r="F5" s="3">
+        <f>1/G5*1000</f>
+        <v>50</v>
+      </c>
+      <c r="G5" s="3">
+        <v>20</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I5" s="3">
+        <v>20</v>
+      </c>
+      <c r="J5" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="K5" s="3">
+        <v>50</v>
+      </c>
+      <c r="L5" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="M5" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="N5" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="U5" s="5"/>
       <c r="V5" s="5"/>
       <c r="W5" s="5"/>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" ht="126" x14ac:dyDescent="0.25">
+      <c r="A6" s="3">
+        <v>5</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="3">
+        <v>0</v>
+      </c>
+      <c r="E6" s="3">
+        <v>250</v>
+      </c>
+      <c r="F6" s="3">
+        <f>1/G6*1000</f>
+        <v>50</v>
+      </c>
+      <c r="G6" s="3">
+        <v>20</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="I6" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="J6" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="K6" s="3">
+        <v>50</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="M6" s="3" t="s">
+        <v>24</v>
+      </c>
+      <c r="N6" s="4" t="s">
+        <v>37</v>
+      </c>
       <c r="O6" s="6"/>
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
@@ -7481,25 +7622,30 @@
       <c r="Y14" s="6"/>
       <c r="Z14" s="6"/>
     </row>
-    <row r="18" spans="13:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="4:13" x14ac:dyDescent="0.25">
       <c r="M18" s="4"/>
+    </row>
+    <row r="20" spans="4:13" ht="283.5" x14ac:dyDescent="0.25">
+      <c r="D20" s="4" t="s">
+        <v>40</v>
+      </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <dataValidations count="5">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2:W1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="U2:W1048576" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"'+x,'-x,'+y,'-y,'+z,'-z"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:M1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="M2:M1048576" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Coordinate excel file, Parameters on the right"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="H2:H1048576" xr:uid="{00000000-0002-0000-0000-000002000000}">
       <formula1>"SC - Global power [mW] (fill in 'Corresponding value'),IGT - Max. pressure in free water [MPa] (fill in 'Corresponding value'),IGT - Voltage [V] (fill in 'Corresponding value'), IGT - Amplitude [%] (fill in 'Corresponding value'),"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:C1048576" xr:uid="{00000000-0002-0000-0000-000003000000}">
       <formula1>"Rectangular - no ramping,Linear,Tukey,"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J1048576">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="J2:J1048576" xr:uid="{00000000-0002-0000-0000-000004000000}">
       <formula1>"Focus wrt exit plane [mm], Focus wrt mid bowl [mm]"</formula1>
     </dataValidation>
   </dataValidations>
@@ -7510,26 +7656,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9cb83fc2-d77f-46b4-9581-c00b781f61fd">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <TaxCatchAll xmlns="8754a512-6dec-483d-b5c6-7cffcc0d02c1" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100C12600718C676640B862E0AA4EBA4F75" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="1f5b5271ce1c64dd6d8fbb2a683be13c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="9cb83fc2-d77f-46b4-9581-c00b781f61fd" xmlns:ns3="8754a512-6dec-483d-b5c6-7cffcc0d02c1" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3472f45d873750127c69500d0e5c45f1" ns2:_="" ns3:_="">
     <xsd:import namespace="9cb83fc2-d77f-46b4-9581-c00b781f61fd"/>
@@ -7752,10 +7878,41 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="9cb83fc2-d77f-46b4-9581-c00b781f61fd">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <TaxCatchAll xmlns="8754a512-6dec-483d-b5c6-7cffcc0d02c1" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C755C0B-1A1A-4CAB-AAB3-F18FC1BEB5C4}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3099BEFB-1261-4A7B-B1BD-10B30D1875E1}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="9cb83fc2-d77f-46b4-9581-c00b781f61fd"/>
+    <ds:schemaRef ds:uri="8754a512-6dec-483d-b5c6-7cffcc0d02c1"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -7772,20 +7929,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3099BEFB-1261-4A7B-B1BD-10B30D1875E1}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9C755C0B-1A1A-4CAB-AAB3-F18FC1BEB5C4}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="9cb83fc2-d77f-46b4-9581-c00b781f61fd"/>
-    <ds:schemaRef ds:uri="8754a512-6dec-483d-b5c6-7cffcc0d02c1"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>